<commit_message>
feat(automation): add comprehensive MM & LMFM Smoke, Positive and Negative suites with strict defect assertions
</commit_message>
<xml_diff>
--- a/TestData/UITestData.xlsx
+++ b/TestData/UITestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Credential" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,6 @@
     <t>Password</t>
   </si>
   <si>
-    <t>Kuchbhi@123</t>
-  </si>
-  <si>
     <t>Branch Sub-Type</t>
   </si>
   <si>
@@ -135,9 +132,6 @@
     <t>Branch Floor dropdown option</t>
   </si>
   <si>
-    <t>VIJAY</t>
-  </si>
-  <si>
     <t>Suspended GSTIN</t>
   </si>
   <si>
@@ -169,6 +163,12 @@
   </si>
   <si>
     <t>07AACCU0153D1ZU</t>
+  </si>
+  <si>
+    <t>Vijay@123</t>
+  </si>
+  <si>
+    <t>Vijay.kumar</t>
   </si>
 </sst>
 </file>
@@ -550,10 +550,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -593,93 +593,93 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" t="s">
-        <v>8</v>
-      </c>
       <c r="G1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" t="s">
         <v>16</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>17</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>18</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>19</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>20</v>
       </c>
-      <c r="N1" t="s">
-        <v>21</v>
-      </c>
       <c r="O1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q1" t="s">
         <v>38</v>
       </c>
-      <c r="Q1" t="s">
-        <v>40</v>
-      </c>
       <c r="R1" t="s">
+        <v>39</v>
+      </c>
+      <c r="S1" t="s">
         <v>41</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
+        <v>42</v>
+      </c>
+      <c r="U1" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="T1" t="s">
-        <v>44</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D2">
         <v>9237937388</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -697,85 +697,85 @@
         <v>1</v>
       </c>
       <c r="N2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="P2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="R2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="S2" t="s">
+        <v>44</v>
+      </c>
+      <c r="T2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" t="s">
         <v>46</v>
-      </c>
-      <c r="T2" t="s">
-        <v>47</v>
-      </c>
-      <c r="U2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:21">
       <c r="O3" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="P3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:21">
       <c r="O4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:21">
       <c r="O5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:21">
       <c r="O6" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="P6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:21">
       <c r="O7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:21">
       <c r="O8" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:21">
       <c r="O9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:21">
       <c r="O10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:21">
       <c r="O11" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>